<commit_message>
Nouvelles mesures correspondant au nouveau script bash
</commit_message>
<xml_diff>
--- a/RENDU_MESURES.xlsx
+++ b/RENDU_MESURES.xlsx
@@ -17,6 +17,26 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+  <si>
+    <t xml:space="preserve">Lignes de code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projet Opti_tour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projet REST</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -89,12 +109,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -221,11 +245,38 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>4140</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>59</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
ajout de la feuille pour le TCF
</commit_message>
<xml_diff>
--- a/RENDU_MESURES.xlsx
+++ b/RENDU_MESURES.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="LOC" sheetId="1" state="visible" r:id="rId3"/>
@@ -14,6 +14,7 @@
     <sheet name="UFC" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="UFC quicksort" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="MI" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="TCF" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="121">
   <si>
     <t xml:space="preserve">Lignes de code</t>
   </si>
@@ -334,6 +335,60 @@
   </si>
   <si>
     <t xml:space="preserve">- autre fonction : remplir d'abord LOC, CC et Halstead, puis vérifier les références de B3:D3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Facteurs Techniques</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAE Relations Internationales IUT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TCF FINAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sauvegarde et récupération fiables ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nécessite une communication de données ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y a t’il des fonctions de traitement distribué ? (calculs sur le telephone par exemple)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Les performances sont elles critiques ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Environnement existant et lourdement utilisé ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saisie de données en ligne ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saisie sur plusieurs écrans ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fichiers principaux mis a jour en ligne ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrées, sorties, fichiers, requêtes complexes ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Traitement interne complexe ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Code conçu pour être réutilisable ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conversion et installation prévues dans la conception ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Système conçu pour multiples organisations et plateformes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L’application est facile d’utilisation pour les utilisateurs ?</t>
   </si>
 </sst>
 </file>
@@ -420,23 +475,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -460,37 +515,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18A303"/>
+        <a:srgbClr val="18a303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369A3"/>
+        <a:srgbClr val="0369a3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A33E03"/>
+        <a:srgbClr val="a33e03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8E03A3"/>
+        <a:srgbClr val="8e03a3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="C99C00"/>
+        <a:srgbClr val="c99c00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="C9211E"/>
+        <a:srgbClr val="c9211e"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000EE"/>
+        <a:srgbClr val="0000ee"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551A8B"/>
+        <a:srgbClr val="551a8b"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -564,13 +619,12 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -615,8 +669,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman"&amp;12 &amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman"&amp;12 Page &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12 &amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12 Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -627,7 +681,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
   </cols>
@@ -710,7 +764,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L23"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11"/>
@@ -1058,7 +1112,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K15"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.01"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14.79"/>
@@ -1292,8 +1346,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman"&amp;12 &amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman"&amp;12 Page &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12 &amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12 Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -1304,7 +1358,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K15"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.01"/>
   </cols>
@@ -1543,8 +1597,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman"&amp;12 &amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman"&amp;12 Page &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12 &amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12 Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -1555,9 +1609,9 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultColWidth="8.34375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.34375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1653,4 +1707,199 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="29.25"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="C2" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" s="0" t="n">
+        <f aca="false"> 0.65 + 0.01 * SUM(C2:C15)</f>
+        <v>1.14</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>108</v>
+      </c>
+      <c r="C3" s="0" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="C4" s="0" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="C5" s="0" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="C6" s="0" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="C7" s="0" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="C8" s="0" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>114</v>
+      </c>
+      <c r="C9" s="0" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="C10" s="0" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="C11" s="0" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="C12" s="0" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="C13" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="C14" s="0" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="C15" s="0" t="n">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Ajout d'une feuille  pour UFC quicksort
</commit_message>
<xml_diff>
--- a/RENDU_MESURES.xlsx
+++ b/RENDU_MESURES.xlsx
@@ -5,13 +5,14 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="LOC" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="CC" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Halstead" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="UFC" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="UFC quicksort" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="79">
   <si>
     <t xml:space="preserve">Lignes de code</t>
   </si>
@@ -244,23 +245,7 @@
     <t xml:space="preserve">Sous-total</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Score t</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">otal UFC</t>
-    </r>
+    <t xml:space="preserve">Score total UFC</t>
   </si>
   <si>
     <t xml:space="preserve">Entrées Externes</t>
@@ -356,20 +341,8 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -377,11 +350,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -560,7 +541,7 @@
   <dimension ref="A1:G6"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -643,8 +624,8 @@
   <dimension ref="A1:L23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -653,7 +634,7 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -662,7 +643,7 @@
       <c r="C2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
@@ -688,7 +669,7 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B3" s="2" t="n">
@@ -699,7 +680,7 @@
         <f aca="false">COUNTA(D7:D14)</f>
         <v>8</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="D3" s="1" t="n">
         <f aca="false">SUM(B7:B23)</f>
         <v>48</v>
       </c>
@@ -742,13 +723,13 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>31</v>
       </c>
       <c r="E6" s="2" t="s">
@@ -759,16 +740,16 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B7" s="0" t="n">
+      <c r="B7" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E7" s="0" t="n">
+      <c r="E7" s="1" t="n">
         <v>7</v>
       </c>
       <c r="L7" s="2" t="s">
@@ -776,30 +757,30 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B8" s="0" t="n">
+      <c r="B8" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E8" s="0" t="n">
+      <c r="E8" s="1" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B9" s="0" t="n">
+      <c r="B9" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="E9" s="0" t="n">
+      <c r="E9" s="1" t="n">
         <v>6</v>
       </c>
       <c r="L9" s="2" t="s">
@@ -807,16 +788,16 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="0" t="n">
+      <c r="B10" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="D10" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E10" s="0" t="n">
+      <c r="E10" s="1" t="n">
         <v>4</v>
       </c>
       <c r="L10" s="2" t="s">
@@ -824,16 +805,16 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="0" t="n">
+      <c r="B11" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D11" s="0" t="s">
+      <c r="D11" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="E11" s="0" t="n">
+      <c r="E11" s="1" t="n">
         <v>4</v>
       </c>
       <c r="L11" s="2" t="s">
@@ -841,16 +822,16 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B12" s="0" t="n">
+      <c r="B12" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="D12" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E12" s="0" t="n">
+      <c r="E12" s="1" t="n">
         <v>3</v>
       </c>
       <c r="L12" s="2" t="s">
@@ -858,30 +839,30 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B13" s="0" t="n">
+      <c r="B13" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="0" t="s">
+      <c r="D13" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="E13" s="0" t="n">
+      <c r="E13" s="1" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B14" s="0" t="n">
+      <c r="B14" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D14" s="0" t="s">
+      <c r="D14" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E14" s="0" t="n">
+      <c r="E14" s="1" t="n">
         <v>2</v>
       </c>
       <c r="L14" s="2" t="s">
@@ -889,10 +870,10 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B15" s="0" t="n">
+      <c r="B15" s="1" t="n">
         <v>2</v>
       </c>
       <c r="L15" s="2" t="s">
@@ -900,10 +881,10 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B16" s="0" t="n">
+      <c r="B16" s="1" t="n">
         <v>2</v>
       </c>
       <c r="L16" s="2" t="s">
@@ -911,10 +892,10 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B17" s="0" t="n">
+      <c r="B17" s="1" t="n">
         <v>2</v>
       </c>
       <c r="L17" s="2" t="s">
@@ -922,10 +903,10 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B18" s="0" t="n">
+      <c r="B18" s="1" t="n">
         <v>1</v>
       </c>
       <c r="L18" s="2" t="s">
@@ -933,42 +914,42 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B19" s="0" t="n">
+      <c r="B19" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B20" s="0" t="n">
+      <c r="B20" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B21" s="0" t="n">
+      <c r="B21" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+      <c r="A22" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B22" s="0" t="n">
+      <c r="B22" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B23" s="0" t="n">
+      <c r="B23" s="1" t="n">
         <v>1</v>
       </c>
     </row>
@@ -991,185 +972,393 @@
   <dimension ref="A1:I7"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14.79"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4"/>
-      <c r="C1" s="4" t="s">
+      <c r="A1" s="1"/>
+      <c r="C1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="1" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="2" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="E3" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="F3" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="G3" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="H3" s="1" t="n">
         <f aca="false">(B3*E3)+(C3*F3)+(D3*G3)</f>
         <v>30</v>
       </c>
-      <c r="I3" s="0" t="n">
+      <c r="I3" s="1" t="n">
         <f aca="false">H3+H4+H5+H6+H7</f>
         <v>144</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="E4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="4" t="n">
+      <c r="E4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="G4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="H4" s="1" t="n">
         <f aca="false">(B4*E4)+(C4*F4)+(D4*G4)</f>
         <v>17</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="F5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="4" t="n">
+      <c r="F5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="1" t="n">
         <f aca="false">(B5*E5)+(C5*F5)+(D5*G5)</f>
         <v>21</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="1" t="n">
         <v>15</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="4" t="n">
+      <c r="F6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="1" t="n">
         <f aca="false">(B6*E6)+(C6*F6)+(D6*G6)</f>
         <v>21</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="E7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="4" t="n">
+      <c r="E7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="G7" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="H7" s="1" t="n">
         <f aca="false">(B7*E7)+(C7*F7)+(D7*G7)</f>
         <v>55</v>
       </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.01"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1"/>
+      <c r="C1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="I1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="1" t="n">
+        <f aca="false">(B3*E3)+(C3*F3)+(D3*G3)</f>
+        <v>6</v>
+      </c>
+      <c r="I3" s="1" t="n">
+        <f aca="false">H3+H4+H5+H6+H7</f>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="1" t="n">
+        <f aca="false">(B4*E4)+(C4*F4)+(D4*G4)</f>
+        <v>4</v>
+      </c>
+      <c r="I4" s="1"/>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="1" t="n">
+        <f aca="false">(B5*E5)+(C5*F5)+(D5*G5)</f>
+        <v>3</v>
+      </c>
+      <c r="I5" s="1"/>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="1" t="n">
+        <f aca="false">(B6*E6)+(C6*F6)+(D6*G6)</f>
+        <v>0</v>
+      </c>
+      <c r="I6" s="1"/>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="1" t="n">
+        <f aca="false">(B7*E7)+(C7*F7)+(D7*G7)</f>
+        <v>0</v>
+      </c>
+      <c r="I7" s="1"/>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E8" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>